<commit_message>
New Files added and Some Removed
</commit_message>
<xml_diff>
--- a/stad_MyPractice/src/test/resources/excel_File/MyPracticeExcel.xlsx
+++ b/stad_MyPractice/src/test/resources/excel_File/MyPracticeExcel.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
   <si>
     <t>SrNo</t>
   </si>
@@ -180,7 +180,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -191,6 +191,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="true"/>
   </cellXfs>
   <cellStyles count="1">
@@ -506,7 +507,7 @@
       <c r="C2" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="5" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>